<commit_message>
Weekly data update: 2026-08-01
</commit_message>
<xml_diff>
--- a/data/financial_metrics_real.xlsx
+++ b/data/financial_metrics_real.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_Metrics" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AMD_Metrics" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM_Metrics" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOOG_Metrics" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVDA_Metrics" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RH_Metrics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPCX_Metrics" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TSLA_Metrics" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Companies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Filings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="All_Metrics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AMD_Metrics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CRM_Metrics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="GOOG_Metrics" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NVDA_Metrics" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="RH_Metrics" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SPCX_Metrics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TSLA_Metrics" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +469,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:54</t>
+          <t>2026-08-01 15:28:21</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:55</t>
+          <t>2026-08-01 15:28:22</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:57</t>
+          <t>2026-08-01 15:28:24</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:58</t>
+          <t>2026-08-01 15:28:25</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:59</t>
+          <t>2026-08-01 15:28:26</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:00</t>
+          <t>2026-08-01 15:28:27</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:01</t>
+          <t>2026-08-01 15:28:28</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:54</t>
+          <t>2026-08-01 15:28:21</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:54</t>
+          <t>2026-08-01 15:28:21</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:54</t>
+          <t>2026-08-01 15:28:21</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:54</t>
+          <t>2026-08-01 15:28:21</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:54</t>
+          <t>2026-08-01 15:28:21</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:55</t>
+          <t>2026-08-01 15:28:22</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:55</t>
+          <t>2026-08-01 15:28:22</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:55</t>
+          <t>2026-08-01 15:28:22</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:55</t>
+          <t>2026-08-01 15:28:22</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:55</t>
+          <t>2026-08-01 15:28:22</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:57</t>
+          <t>2026-08-01 15:28:24</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:57</t>
+          <t>2026-08-01 15:28:24</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:57</t>
+          <t>2026-08-01 15:28:24</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:57</t>
+          <t>2026-08-01 15:28:24</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:58</t>
+          <t>2026-08-01 15:28:25</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:58</t>
+          <t>2026-08-01 15:28:25</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:58</t>
+          <t>2026-08-01 15:28:25</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:58</t>
+          <t>2026-08-01 15:28:25</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:58</t>
+          <t>2026-08-01 15:28:25</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:59</t>
+          <t>2026-08-01 15:28:26</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:59</t>
+          <t>2026-08-01 15:28:26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:59</t>
+          <t>2026-08-01 15:28:26</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:59</t>
+          <t>2026-08-01 15:28:26</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-08-01 00:00:59</t>
+          <t>2026-08-01 15:28:26</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:00</t>
+          <t>2026-08-01 15:28:27</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:00</t>
+          <t>2026-08-01 15:28:27</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:00</t>
+          <t>2026-08-01 15:28:27</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:01</t>
+          <t>2026-08-01 15:28:28</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:01</t>
+          <t>2026-08-01 15:28:28</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:01</t>
+          <t>2026-08-01 15:28:28</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:01</t>
+          <t>2026-08-01 15:28:28</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-01 00:01:01</t>
+          <t>2026-08-01 15:28:28</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">

</xml_diff>

<commit_message>
Add SPCX operating-segment revenue breakdown
Store Connectivity (Starlink), Space (launches), and AI/Other segment
mix in data/segment_metrics.json, load it into a new segment_metrics
table after Yahoo Finance populate, and surface it in chatbot answers,
company profiles, the DB browser, and Excel export.

Co-authored-by: hvelichety <hvelichety@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/financial_metrics_real.xlsx
+++ b/data/financial_metrics_real.xlsx
@@ -10,13 +10,14 @@
     <sheet name="Companies" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Filings" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="All_Metrics" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AMD_Metrics" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CRM_Metrics" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="GOOG_Metrics" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="NVDA_Metrics" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="RH_Metrics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="SPCX_Metrics" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TSLA_Metrics" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Segments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="AMD_Metrics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CRM_Metrics" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="GOOG_Metrics" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="NVDA_Metrics" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="RH_Metrics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SPCX_Metrics" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TSLA_Metrics" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -610,6 +611,392 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Z4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>filing_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>filing_date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>revenue_growth</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>gross_profit</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>operating_income</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>net_income</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>gross_margin</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>operating_margin</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>net_margin</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>total_assets</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>total_liabilities</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>stockholders_equity</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>cash_and_equivalents</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>total_debt</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>operating_cash_flow</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>free_cash_flow</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>capex</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>book_value_per_share</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>research_and_development</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sales_and_marketing</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>employee_count</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>market_cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>18674000000</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>9223000000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-2064000000</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-4937000000</v>
+      </c>
+      <c r="I2" t="n">
+        <v>4427000000</v>
+      </c>
+      <c r="J2" t="n">
+        <v>49.38952554353646</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-11.052800685445</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-26.43782799614437</v>
+      </c>
+      <c r="M2" t="n">
+        <v>92079000000</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50754000000</v>
+      </c>
+      <c r="O2" t="n">
+        <v>41325000000</v>
+      </c>
+      <c r="P2" t="n">
+        <v>24747000000</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>23318000000</v>
+      </c>
+      <c r="R2" t="n">
+        <v>6785000000</v>
+      </c>
+      <c r="S2" t="n">
+        <v>-14121000000</v>
+      </c>
+      <c r="T2" t="n">
+        <v>20906000000</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-0.6520593323835278</v>
+      </c>
+      <c r="V2" t="n">
+        <v>5.458041707666455</v>
+      </c>
+      <c r="W2" t="n">
+        <v>8643000000</v>
+      </c>
+      <c r="X2" t="n">
+        <v>2644000000</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>22000</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1427686686720</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>14015000000</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>6019000000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>742000000</v>
+      </c>
+      <c r="H3" t="n">
+        <v>791000000</v>
+      </c>
+      <c r="I3" t="n">
+        <v>5646000000</v>
+      </c>
+      <c r="J3" t="n">
+        <v>42.94684266856939</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5.29432750624331</v>
+      </c>
+      <c r="L3" t="n">
+        <v>5.643952907599001</v>
+      </c>
+      <c r="M3" t="n">
+        <v>57062000000</v>
+      </c>
+      <c r="N3" t="n">
+        <v>31258000000</v>
+      </c>
+      <c r="O3" t="n">
+        <v>25804000000</v>
+      </c>
+      <c r="P3" t="n">
+        <v>11385000000</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>14175000000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>5776000000</v>
+      </c>
+      <c r="S3" t="n">
+        <v>-5387000000</v>
+      </c>
+      <c r="T3" t="n">
+        <v>11163000000</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.1044721352876991</v>
+      </c>
+      <c r="V3" t="n">
+        <v>3.408089733203271</v>
+      </c>
+      <c r="W3" t="n">
+        <v>3464000000</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1813000000</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>22000</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1427686686720</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2023-12-31</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>10387000000</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>4277000000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>507000000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-4628000000</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-663000000</v>
+      </c>
+      <c r="J4" t="n">
+        <v>41.17647058823529</v>
+      </c>
+      <c r="K4" t="n">
+        <v>4.881101376720901</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-44.55569461827284</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="n">
+        <v>4520000000</v>
+      </c>
+      <c r="S4" t="n">
+        <v>105000000</v>
+      </c>
+      <c r="T4" t="n">
+        <v>4415000000</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-0.6112478408488894</v>
+      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="n">
+        <v>2105000000</v>
+      </c>
+      <c r="X4" t="n">
+        <v>1665000000</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>22000</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>1427686686720</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -19089,6 +19476,196 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>filing_date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>segment_key</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>segment_name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>revenue_share_pct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>profitability_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Space Exploration Technologies Corp.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>connectivity</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Connectivity (Starlink)</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>11400000000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>61</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>profitable</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Starlink consumer, business, maritime, aviation, and government (Starshield). Primary cash-flow engine with recurring subscription revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Space Exploration Technologies Corp.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>space</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Space (Launch Services)</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4100000000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>22</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>near_breakeven</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Commercial, NASA, and DoD launches (Falcon 9, Falcon Heavy, Starship). Many Falcon 9 flights are internal Starlink deployments, so external launch revenue is lower than total launch activity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Space Exploration Technologies Corp.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ai_other</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AI / Other</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>3200000000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>17</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>loss_making</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AI products, compute, and related activities (xAI-related, Grok, X, compute infrastructure). Heavily loss-making due to compute and development spend.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -19583,7 +20160,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20083,7 +20660,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20557,7 +21134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21075,7 +21652,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21591,390 +22168,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Z4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>filing_type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>filing_date</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>total_revenue</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>revenue_growth</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>gross_profit</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>operating_income</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>net_income</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>ebitda</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>gross_margin</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>operating_margin</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>net_margin</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>total_assets</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>total_liabilities</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>stockholders_equity</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>cash_and_equivalents</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>total_debt</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>operating_cash_flow</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>capex</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>eps</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>book_value_per_share</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>research_and_development</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>sales_and_marketing</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>employee_count</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>market_cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SPCX</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2025-12-31</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>18674000000</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
-        <v>9223000000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-2064000000</v>
-      </c>
-      <c r="H2" t="n">
-        <v>-4937000000</v>
-      </c>
-      <c r="I2" t="n">
-        <v>4427000000</v>
-      </c>
-      <c r="J2" t="n">
-        <v>49.38952554353646</v>
-      </c>
-      <c r="K2" t="n">
-        <v>-11.052800685445</v>
-      </c>
-      <c r="L2" t="n">
-        <v>-26.43782799614437</v>
-      </c>
-      <c r="M2" t="n">
-        <v>92079000000</v>
-      </c>
-      <c r="N2" t="n">
-        <v>50754000000</v>
-      </c>
-      <c r="O2" t="n">
-        <v>41325000000</v>
-      </c>
-      <c r="P2" t="n">
-        <v>24747000000</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>23318000000</v>
-      </c>
-      <c r="R2" t="n">
-        <v>6785000000</v>
-      </c>
-      <c r="S2" t="n">
-        <v>-14121000000</v>
-      </c>
-      <c r="T2" t="n">
-        <v>20906000000</v>
-      </c>
-      <c r="U2" t="n">
-        <v>-0.6520593323835278</v>
-      </c>
-      <c r="V2" t="n">
-        <v>5.458041707666455</v>
-      </c>
-      <c r="W2" t="n">
-        <v>8643000000</v>
-      </c>
-      <c r="X2" t="n">
-        <v>2644000000</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1427686686720</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SPCX</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2024-12-31</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>14015000000</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="n">
-        <v>6019000000</v>
-      </c>
-      <c r="G3" t="n">
-        <v>742000000</v>
-      </c>
-      <c r="H3" t="n">
-        <v>791000000</v>
-      </c>
-      <c r="I3" t="n">
-        <v>5646000000</v>
-      </c>
-      <c r="J3" t="n">
-        <v>42.94684266856939</v>
-      </c>
-      <c r="K3" t="n">
-        <v>5.29432750624331</v>
-      </c>
-      <c r="L3" t="n">
-        <v>5.643952907599001</v>
-      </c>
-      <c r="M3" t="n">
-        <v>57062000000</v>
-      </c>
-      <c r="N3" t="n">
-        <v>31258000000</v>
-      </c>
-      <c r="O3" t="n">
-        <v>25804000000</v>
-      </c>
-      <c r="P3" t="n">
-        <v>11385000000</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>14175000000</v>
-      </c>
-      <c r="R3" t="n">
-        <v>5776000000</v>
-      </c>
-      <c r="S3" t="n">
-        <v>-5387000000</v>
-      </c>
-      <c r="T3" t="n">
-        <v>11163000000</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.1044721352876991</v>
-      </c>
-      <c r="V3" t="n">
-        <v>3.408089733203271</v>
-      </c>
-      <c r="W3" t="n">
-        <v>3464000000</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1813000000</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1427686686720</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SPCX</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2023-12-31</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>10387000000</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="n">
-        <v>4277000000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>507000000</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-4628000000</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-663000000</v>
-      </c>
-      <c r="J4" t="n">
-        <v>41.17647058823529</v>
-      </c>
-      <c r="K4" t="n">
-        <v>4.881101376720901</v>
-      </c>
-      <c r="L4" t="n">
-        <v>-44.55569461827284</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="n">
-        <v>4520000000</v>
-      </c>
-      <c r="S4" t="n">
-        <v>105000000</v>
-      </c>
-      <c r="T4" t="n">
-        <v>4415000000</v>
-      </c>
-      <c r="U4" t="n">
-        <v>-0.6112478408488894</v>
-      </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="n">
-        <v>2105000000</v>
-      </c>
-      <c r="X4" t="n">
-        <v>1665000000</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>1427686686720</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>